<commit_message>
Checklist de Projeto para Elaboração feito
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/BRA - Checklist Verificacao de Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/BRA - Checklist Verificacao de Projeto.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0C6817-34FD-4E10-8215-AE31183EBF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0EB288C-68B1-4AB8-A090-6EB4E34D0C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="666" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="666" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicadores" sheetId="6" r:id="rId1"/>
@@ -710,7 +710,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="123">
   <si>
     <t>Ambiente</t>
   </si>
@@ -1067,6 +1067,18 @@
   </si>
   <si>
     <t>Fábio Adriano Silveira</t>
+  </si>
+  <si>
+    <t>Parcialmente</t>
+  </si>
+  <si>
+    <t>Implementação e testes desenvolvidos, testes não registrados</t>
+  </si>
+  <si>
+    <t>Modelo de Implementação não definido</t>
+  </si>
+  <si>
+    <t>Executados mas não registrados</t>
   </si>
 </sst>
 </file>
@@ -1471,6 +1483,9 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -1521,9 +1536,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1631,7 +1643,7 @@
                   <c:v>0.95238095238095233</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.76</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2591,13 +2603,13 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -2606,22 +2618,22 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>0.66666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2710,7 +2722,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -2719,13 +2731,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.4</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -2734,7 +2746,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2939,7 +2951,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2954,7 +2966,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -7320,10 +7332,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="41"/>
+      <c r="B1" s="42"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="18" t="s">
@@ -7346,9 +7358,9 @@
       <c r="A4" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="20" t="e">
+      <c r="B4" s="20">
         <f>'Ver-Elaboração1'!$F$2</f>
-        <v>#DIV/0!</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -7451,21 +7463,21 @@
       <c r="N2" t="s">
         <v>2</v>
       </c>
-      <c r="O2" s="25" t="e">
+      <c r="O2" s="25">
         <f>('Ver-Elaboração1'!$G$6/SUM('Ver-Elaboração1'!$G$6:'Ver-Elaboração1'!$J$6))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P2" s="25" t="e">
+        <v>1</v>
+      </c>
+      <c r="P2" s="25">
         <f>('Ver-Elaboração1'!$H$6/SUM('Ver-Elaboração1'!$G$6:'Ver-Elaboração1'!$J$6))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q2" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="25">
         <f>('Ver-Elaboração1'!$I$6/SUM('Ver-Elaboração1'!$G$6:'Ver-Elaboração1'!$J$6))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R2" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R2" s="25">
         <f>('Ver-Elaboração1'!$J$6/SUM('Ver-Elaboração1'!$G$6:'Ver-Elaboração1'!$J$6))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -7491,21 +7503,21 @@
       <c r="N3" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="25" t="e">
+      <c r="O3" s="25">
         <f>('Ver-Elaboração1'!$G$8/SUM('Ver-Elaboração1'!$G$8:'Ver-Elaboração1'!$J$8))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P3" s="25" t="e">
+        <v>1</v>
+      </c>
+      <c r="P3" s="25">
         <f>('Ver-Elaboração1'!$H$8/SUM('Ver-Elaboração1'!$G$8:'Ver-Elaboração1'!$J$8))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q3" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="25">
         <f>('Ver-Elaboração1'!$I$8/SUM('Ver-Elaboração1'!$G$8:'Ver-Elaboração1'!$J$8))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R3" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R3" s="25">
         <f>('Ver-Elaboração1'!$J$8/SUM('Ver-Elaboração1'!$G$8:'Ver-Elaboração1'!$J$8))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -7531,21 +7543,21 @@
       <c r="N4" t="s">
         <v>14</v>
       </c>
-      <c r="O4" s="25" t="e">
+      <c r="O4" s="25">
         <f>('Ver-Elaboração1'!$G$11/SUM('Ver-Elaboração1'!$G$11:'Ver-Elaboração1'!$J$11))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P4" s="25" t="e">
+        <v>0.75</v>
+      </c>
+      <c r="P4" s="25">
         <f>('Ver-Elaboração1'!$H$11/SUM('Ver-Elaboração1'!$G$11:'Ver-Elaboração1'!$J$11))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q4" s="25" t="e">
+        <v>0.25</v>
+      </c>
+      <c r="Q4" s="25">
         <f>('Ver-Elaboração1'!$I$11/SUM('Ver-Elaboração1'!$G$11:'Ver-Elaboração1'!$J$11))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R4" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R4" s="25">
         <f>('Ver-Elaboração1'!$J$11/SUM('Ver-Elaboração1'!$G$11:'Ver-Elaboração1'!$J$11))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:18">
@@ -7571,21 +7583,21 @@
       <c r="N5" t="s">
         <v>4</v>
       </c>
-      <c r="O5" s="25" t="e">
+      <c r="O5" s="25">
         <f>('Ver-Elaboração1'!$G$16/SUM('Ver-Elaboração1'!$G$16:'Ver-Elaboração1'!$J$16))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P5" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="P5" s="25">
         <f>('Ver-Elaboração1'!$H$16/SUM('Ver-Elaboração1'!$G$16:'Ver-Elaboração1'!$J$16))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q5" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="25">
         <f>('Ver-Elaboração1'!$I$16/SUM('Ver-Elaboração1'!$G$16:'Ver-Elaboração1'!$J$16))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R5" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R5" s="25">
         <f>('Ver-Elaboração1'!$J$16/SUM('Ver-Elaboração1'!$G$16:'Ver-Elaboração1'!$J$16))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:18">
@@ -7651,21 +7663,21 @@
       <c r="N7" t="s">
         <v>5</v>
       </c>
-      <c r="O7" s="25" t="e">
+      <c r="O7" s="25">
         <f>('Ver-Elaboração1'!$G$18/SUM('Ver-Elaboração1'!$G$18:'Ver-Elaboração1'!$J$18))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P7" s="25" t="e">
+        <v>0.5</v>
+      </c>
+      <c r="P7" s="25">
         <f>('Ver-Elaboração1'!$H$18/SUM('Ver-Elaboração1'!$G$18:'Ver-Elaboração1'!$J$18))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q7" s="25" t="e">
+        <v>0.5</v>
+      </c>
+      <c r="Q7" s="25">
         <f>('Ver-Elaboração1'!$I$18/SUM('Ver-Elaboração1'!$G$18:'Ver-Elaboração1'!$J$18))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R7" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R7" s="25">
         <f>('Ver-Elaboração1'!$J$18/SUM('Ver-Elaboração1'!$G$18:'Ver-Elaboração1'!$J$18))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -7731,21 +7743,21 @@
       <c r="N9" t="s">
         <v>6</v>
       </c>
-      <c r="O9" s="25" t="e">
+      <c r="O9" s="25">
         <f>('Ver-Elaboração1'!$G$23/SUM('Ver-Elaboração1'!$G$23:'Ver-Elaboração1'!$J$23))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P9" s="25" t="e">
+        <v>0.6</v>
+      </c>
+      <c r="P9" s="25">
         <f>('Ver-Elaboração1'!$H$23/SUM('Ver-Elaboração1'!$G$23:'Ver-Elaboração1'!$J$23))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q9" s="25" t="e">
+        <v>0.4</v>
+      </c>
+      <c r="Q9" s="25">
         <f>('Ver-Elaboração1'!$I$23/SUM('Ver-Elaboração1'!$G$23:'Ver-Elaboração1'!$J$23))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R9" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R9" s="25">
         <f>('Ver-Elaboração1'!$J$23/SUM('Ver-Elaboração1'!$G$23:'Ver-Elaboração1'!$J$23))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:18">
@@ -7771,21 +7783,21 @@
       <c r="N10" t="s">
         <v>13</v>
       </c>
-      <c r="O10" s="25" t="e">
+      <c r="O10" s="25">
         <f>('Ver-Elaboração1'!$G$29/SUM('Ver-Elaboração1'!$G$29:'Ver-Elaboração1'!$J$29))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P10" s="25" t="e">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="P10" s="25">
         <f>('Ver-Elaboração1'!$H$29/SUM('Ver-Elaboração1'!$G$29:'Ver-Elaboração1'!$J$29))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q10" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="25">
         <f>('Ver-Elaboração1'!$I$29/SUM('Ver-Elaboração1'!$G$29:'Ver-Elaboração1'!$J$29))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R10" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R10" s="25">
         <f>('Ver-Elaboração1'!$J$29/SUM('Ver-Elaboração1'!$G$29:'Ver-Elaboração1'!$J$29))</f>
-        <v>#DIV/0!</v>
+        <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="11" spans="1:18">
@@ -7811,21 +7823,21 @@
       <c r="N11" t="s">
         <v>56</v>
       </c>
-      <c r="O11" s="25" t="e">
+      <c r="O11" s="25">
         <f>('Ver-Elaboração1'!$G$36/SUM('Ver-Elaboração1'!$G$36:'Ver-Elaboração1'!$J$36))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P11" s="25" t="e">
+        <v>1</v>
+      </c>
+      <c r="P11" s="25">
         <f>('Ver-Elaboração1'!$H$36/SUM('Ver-Elaboração1'!$G$36:'Ver-Elaboração1'!$J$36))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q11" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="25">
         <f>('Ver-Elaboração1'!$I$36/SUM('Ver-Elaboração1'!$G$36:'Ver-Elaboração1'!$J$36))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R11" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R11" s="25">
         <f>('Ver-Elaboração1'!$J$36/SUM('Ver-Elaboração1'!$G$36:'Ver-Elaboração1'!$J$36))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:18">
@@ -7851,21 +7863,21 @@
       <c r="N12" t="s">
         <v>15</v>
       </c>
-      <c r="O12" s="25" t="e">
+      <c r="O12" s="25">
         <f>('Ver-Elaboração1'!$G$40/SUM('Ver-Elaboração1'!$G$40:'Ver-Elaboração1'!$J$40))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P12" s="25" t="e">
+        <v>0.5</v>
+      </c>
+      <c r="P12" s="25">
         <f>('Ver-Elaboração1'!$H$40/SUM('Ver-Elaboração1'!$G$40:'Ver-Elaboração1'!$J$40))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q12" s="25" t="e">
+        <v>0.5</v>
+      </c>
+      <c r="Q12" s="25">
         <f>('Ver-Elaboração1'!$I$40/SUM('Ver-Elaboração1'!$G$40:'Ver-Elaboração1'!$J$40))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R12" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R12" s="25">
         <f>('Ver-Elaboração1'!$J$40/SUM('Ver-Elaboração1'!$G$40:'Ver-Elaboração1'!$J$40))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:17">
@@ -8432,45 +8444,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="33"/>
+      <c r="B2" s="34"/>
       <c r="C2" s="28">
         <v>46259</v>
       </c>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="40"/>
+      <c r="E2" s="41"/>
       <c r="F2" s="21">
         <f>COUNTIF(D5:D41,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
         <v>0.95238095238095233</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="33"/>
+      <c r="B3" s="34"/>
       <c r="C3" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="37"/>
-      <c r="F3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="39"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -8493,7 +8505,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="14.4">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="9"/>
@@ -8521,7 +8533,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="35"/>
+      <c r="A6" s="36"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -8535,7 +8547,7 @@
       <c r="F6" s="8"/>
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="35" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="9"/>
@@ -8563,7 +8575,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" ht="15" customHeight="1">
-      <c r="A8" s="31"/>
+      <c r="A8" s="32"/>
       <c r="B8" s="22">
         <v>2</v>
       </c>
@@ -8577,7 +8589,7 @@
       <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:10" ht="14.4">
-      <c r="A9" s="31"/>
+      <c r="A9" s="32"/>
       <c r="B9" s="5">
         <v>3</v>
       </c>
@@ -8591,7 +8603,7 @@
       <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:10" ht="14.4">
-      <c r="A10" s="31"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="5">
         <v>4</v>
       </c>
@@ -8605,7 +8617,7 @@
       <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:10" s="1" customFormat="1" ht="14.4">
-      <c r="A11" s="31"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="5">
         <v>5</v>
       </c>
@@ -8619,7 +8631,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="16.5" customHeight="1">
-      <c r="A12" s="31"/>
+      <c r="A12" s="32"/>
       <c r="B12" s="5">
         <v>6</v>
       </c>
@@ -8633,7 +8645,7 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="31"/>
+      <c r="A13" s="32"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>3</v>
@@ -8659,7 +8671,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="14.4">
-      <c r="A14" s="31"/>
+      <c r="A14" s="32"/>
       <c r="B14" s="23">
         <v>7</v>
       </c>
@@ -8673,7 +8685,7 @@
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A15" s="31"/>
+      <c r="A15" s="32"/>
       <c r="B15" s="5">
         <v>8</v>
       </c>
@@ -8687,7 +8699,7 @@
       <c r="F15" s="8"/>
     </row>
     <row r="16" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A16" s="31"/>
+      <c r="A16" s="32"/>
       <c r="B16" s="5">
         <v>9</v>
       </c>
@@ -8701,7 +8713,7 @@
       <c r="F16" s="8"/>
     </row>
     <row r="17" spans="1:10" s="1" customFormat="1" ht="14.4">
-      <c r="A17" s="31"/>
+      <c r="A17" s="32"/>
       <c r="B17" s="23">
         <v>10</v>
       </c>
@@ -8715,7 +8727,7 @@
       <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:10" s="1" customFormat="1" ht="14.4">
-      <c r="A18" s="31"/>
+      <c r="A18" s="32"/>
       <c r="B18" s="5">
         <v>11</v>
       </c>
@@ -8729,7 +8741,7 @@
       <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:10" ht="14.4">
-      <c r="A19" s="31"/>
+      <c r="A19" s="32"/>
       <c r="B19" s="9"/>
       <c r="C19" s="10" t="s">
         <v>97</v>
@@ -8755,7 +8767,7 @@
       </c>
     </row>
     <row r="20" spans="1:10" ht="14.4">
-      <c r="A20" s="31"/>
+      <c r="A20" s="32"/>
       <c r="B20" s="23">
         <v>12</v>
       </c>
@@ -8769,7 +8781,7 @@
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="28.8">
-      <c r="A21" s="31"/>
+      <c r="A21" s="32"/>
       <c r="B21" s="5">
         <v>13</v>
       </c>
@@ -8783,7 +8795,7 @@
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="31"/>
+      <c r="A22" s="32"/>
       <c r="B22" s="9"/>
       <c r="C22" s="10" t="s">
         <v>4</v>
@@ -8809,7 +8821,7 @@
       </c>
     </row>
     <row r="23" spans="1:10" ht="14.4">
-      <c r="A23" s="31"/>
+      <c r="A23" s="32"/>
       <c r="B23" s="23">
         <v>14</v>
       </c>
@@ -8823,7 +8835,7 @@
       <c r="F23" s="8"/>
     </row>
     <row r="24" spans="1:10" ht="14.4">
-      <c r="A24" s="31"/>
+      <c r="A24" s="32"/>
       <c r="B24" s="5">
         <v>15</v>
       </c>
@@ -8837,7 +8849,7 @@
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:10" ht="14.4">
-      <c r="A25" s="31"/>
+      <c r="A25" s="32"/>
       <c r="B25" s="9"/>
       <c r="C25" s="10" t="s">
         <v>36</v>
@@ -8863,7 +8875,7 @@
       </c>
     </row>
     <row r="26" spans="1:10" ht="14.4">
-      <c r="A26" s="31"/>
+      <c r="A26" s="32"/>
       <c r="B26" s="23">
         <v>16</v>
       </c>
@@ -8877,7 +8889,7 @@
       <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:10" ht="14.4">
-      <c r="A27" s="31"/>
+      <c r="A27" s="32"/>
       <c r="B27" s="5">
         <v>17</v>
       </c>
@@ -8891,7 +8903,7 @@
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="31"/>
+      <c r="A28" s="32"/>
       <c r="B28" s="9"/>
       <c r="C28" s="10" t="s">
         <v>13</v>
@@ -8917,7 +8929,7 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="14.4">
-      <c r="A29" s="31"/>
+      <c r="A29" s="32"/>
       <c r="B29" s="23">
         <v>21</v>
       </c>
@@ -8931,7 +8943,7 @@
       <c r="F29" s="8"/>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="31"/>
+      <c r="A30" s="32"/>
       <c r="B30" s="5">
         <v>22</v>
       </c>
@@ -8945,7 +8957,7 @@
       <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:10" ht="14.4">
-      <c r="A31" s="31"/>
+      <c r="A31" s="32"/>
       <c r="B31" s="5">
         <v>23</v>
       </c>
@@ -8959,7 +8971,7 @@
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="14.4">
-      <c r="A32" s="31"/>
+      <c r="A32" s="32"/>
       <c r="B32" s="5">
         <v>24</v>
       </c>
@@ -8973,7 +8985,7 @@
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="31"/>
+      <c r="A33" s="32"/>
       <c r="B33" s="5">
         <v>25</v>
       </c>
@@ -8987,7 +8999,7 @@
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="31"/>
+      <c r="A34" s="32"/>
       <c r="B34" s="5">
         <v>26</v>
       </c>
@@ -9000,7 +9012,7 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="18.75" customHeight="1">
-      <c r="A35" s="31"/>
+      <c r="A35" s="32"/>
       <c r="B35" s="5">
         <v>27</v>
       </c>
@@ -9014,21 +9026,21 @@
       <c r="F35" s="8"/>
     </row>
     <row r="36" spans="1:10" ht="14.4">
-      <c r="A36" s="31"/>
+      <c r="A36" s="32"/>
       <c r="B36" s="5">
         <v>28</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D36" s="46" t="s">
+      <c r="D36" s="29" t="s">
         <v>115</v>
       </c>
       <c r="E36" s="8"/>
       <c r="F36" s="8"/>
     </row>
     <row r="37" spans="1:10" ht="15" customHeight="1">
-      <c r="A37" s="29" t="s">
+      <c r="A37" s="30" t="s">
         <v>30</v>
       </c>
       <c r="B37" s="9"/>
@@ -9056,7 +9068,7 @@
       </c>
     </row>
     <row r="38" spans="1:10" ht="14.4">
-      <c r="A38" s="30"/>
+      <c r="A38" s="31"/>
       <c r="B38" s="23">
         <v>30</v>
       </c>
@@ -9070,7 +9082,7 @@
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="14.4">
-      <c r="A39" s="30"/>
+      <c r="A39" s="31"/>
       <c r="B39" s="5">
         <v>31</v>
       </c>
@@ -9084,7 +9096,7 @@
       <c r="F39" s="8"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="30"/>
+      <c r="A40" s="31"/>
       <c r="B40" s="5">
         <v>32</v>
       </c>
@@ -9098,7 +9110,7 @@
       <c r="F40" s="8"/>
     </row>
     <row r="41" spans="1:10" ht="20.25" customHeight="1">
-      <c r="A41" s="30"/>
+      <c r="A41" s="31"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
@@ -9151,41 +9163,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="39" t="s">
+      <c r="B2" s="34"/>
+      <c r="C2" s="28">
+        <v>46323</v>
+      </c>
+      <c r="D2" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="40"/>
-      <c r="F2" s="21" t="e">
+      <c r="E2" s="41"/>
+      <c r="F2" s="21">
         <f>COUNTIF(D5:D41,"Sim")/(COUNTA(D5:D42)-COUNTIF(D5:D42,"NA"))</f>
-        <v>#DIV/0!</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="43" t="s">
+      <c r="B3" s="34"/>
+      <c r="C3" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="44"/>
-      <c r="F3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="46"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -9208,7 +9224,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="35" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -9220,19 +9236,21 @@
       <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="31"/>
+      <c r="A6" s="32"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6">
         <f>COUNTIF(D6,"Sim")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6">
         <f>COUNTIF(D6,"Parcialmente")</f>
@@ -9248,7 +9266,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="14.4">
-      <c r="A7" s="31"/>
+      <c r="A7" s="32"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -9258,19 +9276,21 @@
       <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A8" s="31"/>
+      <c r="A8" s="32"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8">
         <f>COUNTIF(D8,"Sim")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8">
         <f>COUNTIF(D8,"Parcialmente")</f>
@@ -9286,14 +9306,16 @@
       </c>
     </row>
     <row r="9" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A9" s="31"/>
+      <c r="A9" s="32"/>
       <c r="B9" s="5">
         <v>3</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
       <c r="G9"/>
@@ -9302,7 +9324,7 @@
       <c r="J9"/>
     </row>
     <row r="10" spans="1:10" ht="14.4">
-      <c r="A10" s="31"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="9"/>
       <c r="C10" s="10" t="s">
         <v>97</v>
@@ -9312,23 +9334,25 @@
       <c r="F10" s="12"/>
     </row>
     <row r="11" spans="1:10" ht="28.8">
-      <c r="A11" s="31"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="23">
         <v>4</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="D11" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
       <c r="G11">
         <f>COUNTIF(D11:D14,"Sim")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H11">
         <f>COUNTIF(D11:D14,"Parcialmente")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11">
         <f>COUNTIF(D11:D14,"Não")</f>
@@ -9340,43 +9364,49 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="28.8">
-      <c r="A12" s="31"/>
+      <c r="A12" s="32"/>
       <c r="B12" s="23">
         <v>5</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="31"/>
+      <c r="A13" s="32"/>
       <c r="B13" s="5">
         <v>6</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="3"/>
+      <c r="D13" s="3" t="s">
+        <v>119</v>
+      </c>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:10" ht="28.8">
-      <c r="A14" s="31"/>
+      <c r="A14" s="32"/>
       <c r="B14" s="5">
         <v>7</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:10" ht="14.4">
-      <c r="A15" s="31"/>
+      <c r="A15" s="32"/>
       <c r="B15" s="9"/>
       <c r="C15" s="10" t="s">
         <v>4</v>
@@ -9386,14 +9416,16 @@
       <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:10" ht="14.4">
-      <c r="A16" s="31"/>
+      <c r="A16" s="32"/>
       <c r="B16" s="5">
         <v>7</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
       <c r="G16">
@@ -9410,11 +9442,11 @@
       </c>
       <c r="J16">
         <f>COUNTIF(D16,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="35" t="s">
         <v>18</v>
       </c>
       <c r="B17" s="9"/>
@@ -9425,24 +9457,28 @@
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
     </row>
-    <row r="18" spans="1:10" ht="28.8">
-      <c r="A18" s="31"/>
+    <row r="18" spans="1:10" ht="43.2">
+      <c r="A18" s="32"/>
       <c r="B18" s="5">
         <v>9</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="3"/>
-      <c r="E18" s="8"/>
+      <c r="D18" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>120</v>
+      </c>
       <c r="F18" s="8"/>
       <c r="G18">
         <f>COUNTIF(D18:D21,"Sim")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H18">
         <f>COUNTIF(D18:D21,"Parcialmente")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I18">
         <f>COUNTIF(D18:D21,"Não")</f>
@@ -9454,43 +9490,51 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="28.8">
-      <c r="A19" s="31"/>
+      <c r="A19" s="32"/>
       <c r="B19" s="23">
         <v>10</v>
       </c>
       <c r="C19" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="3"/>
-      <c r="E19" s="8"/>
+      <c r="D19" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>121</v>
+      </c>
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A20" s="31"/>
+      <c r="A20" s="32"/>
       <c r="B20" s="5">
         <v>11</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D20" s="3"/>
+      <c r="D20" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="28.8">
-      <c r="A21" s="31"/>
+      <c r="A21" s="32"/>
       <c r="B21" s="5">
         <v>12</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="34" t="s">
+      <c r="A22" s="35" t="s">
         <v>19</v>
       </c>
       <c r="B22" s="9"/>
@@ -9501,24 +9545,28 @@
       <c r="E22" s="12"/>
       <c r="F22" s="12"/>
     </row>
-    <row r="23" spans="1:10" ht="28.8">
-      <c r="A23" s="31"/>
+    <row r="23" spans="1:10" ht="43.2">
+      <c r="A23" s="32"/>
       <c r="B23" s="5">
         <v>17</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D23" s="3"/>
-      <c r="E23" s="8"/>
+      <c r="D23" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>120</v>
+      </c>
       <c r="F23" s="8"/>
       <c r="G23">
         <f>COUNTIF(D23:D27,"Sim")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H23">
         <f>COUNTIF(D23:D27,"Parcialmente")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I23">
         <f>COUNTIF(D23:D27,"Não")</f>
@@ -9530,55 +9578,65 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="28.8">
-      <c r="A24" s="31"/>
+      <c r="A24" s="32"/>
       <c r="B24" s="5">
         <v>18</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D24" s="3"/>
+      <c r="D24" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:10" ht="28.8">
-      <c r="A25" s="31"/>
+      <c r="A25" s="32"/>
       <c r="B25" s="5">
         <v>19</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="D25" s="3"/>
+      <c r="D25" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:10" ht="14.4">
-      <c r="A26" s="31"/>
+      <c r="A26" s="32"/>
       <c r="B26" s="5">
         <v>21</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D26" s="3"/>
+      <c r="D26" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:10" ht="14.4">
-      <c r="A27" s="31"/>
+      <c r="A27" s="32"/>
       <c r="B27" s="5">
         <v>22</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="D27" s="3"/>
-      <c r="E27" s="8"/>
+      <c r="D27" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>122</v>
+      </c>
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="43" t="s">
         <v>11</v>
       </c>
       <c r="B28" s="9"/>
@@ -9590,19 +9648,21 @@
       <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:10" ht="14.4">
-      <c r="A29" s="42"/>
+      <c r="A29" s="43"/>
       <c r="B29" s="5">
         <v>23</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D29" s="3"/>
+      <c r="D29" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E29" s="8"/>
       <c r="F29" s="8"/>
       <c r="G29">
         <f>COUNTIF(D29:D34,"Sim")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H29">
         <f>COUNTIF(D29:D34,"Parcialmente")</f>
@@ -9614,71 +9674,81 @@
       </c>
       <c r="J29">
         <f>COUNTIF(D29:D34,"NA")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="42"/>
+      <c r="A30" s="43"/>
       <c r="B30" s="5">
         <v>24</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D30" s="3"/>
+      <c r="D30" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:10" ht="28.8">
-      <c r="A31" s="42"/>
+      <c r="A31" s="43"/>
       <c r="B31" s="5">
         <v>25</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D31" s="3"/>
+      <c r="D31" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="14.4">
-      <c r="A32" s="42"/>
+      <c r="A32" s="43"/>
       <c r="B32" s="5">
         <v>26</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="D32" s="3"/>
+      <c r="D32" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="42"/>
+      <c r="A33" s="43"/>
       <c r="B33" s="5">
         <v>27</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D33" s="3"/>
+      <c r="D33" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="42"/>
+      <c r="A34" s="43"/>
       <c r="B34" s="5">
         <v>28</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D34" s="3"/>
+      <c r="D34" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1">
-      <c r="A35" s="29" t="s">
+      <c r="A35" s="30" t="s">
         <v>30</v>
       </c>
       <c r="B35" s="9"/>
@@ -9690,19 +9760,21 @@
       <c r="F35" s="12"/>
     </row>
     <row r="36" spans="1:10" ht="28.8">
-      <c r="A36" s="30"/>
+      <c r="A36" s="31"/>
       <c r="B36" s="5">
         <v>29</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D36" s="3"/>
+      <c r="D36" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E36" s="8"/>
       <c r="F36" s="8"/>
       <c r="G36">
         <f>COUNTIF(D36:D38,"Sim")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H36">
         <f>COUNTIF(D36:D38,"Parcialmente")</f>
@@ -9718,31 +9790,35 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="14.4">
-      <c r="A37" s="30"/>
+      <c r="A37" s="31"/>
       <c r="B37" s="5">
         <v>30</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D37" s="3"/>
+      <c r="D37" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E37" s="8"/>
       <c r="F37" s="8"/>
     </row>
     <row r="38" spans="1:10" ht="28.8">
-      <c r="A38" s="30"/>
+      <c r="A38" s="31"/>
       <c r="B38" s="5">
         <v>31</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D38" s="3"/>
+      <c r="D38" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="14.4">
-      <c r="A39" s="30"/>
+      <c r="A39" s="31"/>
       <c r="B39" s="9"/>
       <c r="C39" s="10" t="s">
         <v>15</v>
@@ -9752,23 +9828,25 @@
       <c r="F39" s="12"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="30"/>
+      <c r="A40" s="31"/>
       <c r="B40" s="5">
         <v>32</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D40" s="3"/>
+      <c r="D40" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E40" s="8"/>
       <c r="F40" s="8"/>
       <c r="G40">
         <f>COUNTIF(D40:D41,"Sim")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H40">
         <f>COUNTIF(D40:D41,"Parcialmente")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40">
         <f>COUNTIF(D40:D41,"Não")</f>
@@ -9780,14 +9858,16 @@
       </c>
     </row>
     <row r="41" spans="1:10" ht="14.4">
-      <c r="A41" s="30"/>
+      <c r="A41" s="31"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D41" s="3"/>
+      <c r="D41" s="3" t="s">
+        <v>119</v>
+      </c>
       <c r="E41" s="8"/>
       <c r="F41" s="8"/>
     </row>
@@ -9832,41 +9912,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="33"/>
+      <c r="B2" s="34"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="40"/>
+      <c r="E2" s="41"/>
       <c r="F2" s="21" t="e">
         <f>COUNTIF(D5:D42,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="33"/>
+      <c r="B3" s="34"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="44"/>
-      <c r="F3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="46"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -9889,7 +9969,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="35" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -9901,7 +9981,7 @@
       <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="31"/>
+      <c r="A6" s="32"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -9929,7 +10009,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="14.4">
-      <c r="A7" s="31"/>
+      <c r="A7" s="32"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -9939,7 +10019,7 @@
       <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A8" s="31"/>
+      <c r="A8" s="32"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
@@ -9967,7 +10047,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="14.4">
-      <c r="A9" s="31"/>
+      <c r="A9" s="32"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10" t="s">
         <v>97</v>
@@ -9977,7 +10057,7 @@
       <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:10" ht="28.8">
-      <c r="A10" s="31"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="5">
         <v>3</v>
       </c>
@@ -10005,7 +10085,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.8">
-      <c r="A11" s="31"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="5">
         <v>4</v>
       </c>
@@ -10017,7 +10097,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="18.75" customHeight="1">
-      <c r="A12" s="31"/>
+      <c r="A12" s="32"/>
       <c r="B12" s="5">
         <v>5</v>
       </c>
@@ -10029,7 +10109,7 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="31"/>
+      <c r="A13" s="32"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>4</v>
@@ -10039,7 +10119,7 @@
       <c r="F13" s="12"/>
     </row>
     <row r="14" spans="1:10" ht="14.4">
-      <c r="A14" s="31"/>
+      <c r="A14" s="32"/>
       <c r="B14" s="5">
         <v>6</v>
       </c>
@@ -10067,7 +10147,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1">
-      <c r="A15" s="34" t="s">
+      <c r="A15" s="35" t="s">
         <v>18</v>
       </c>
       <c r="B15" s="9"/>
@@ -10079,7 +10159,7 @@
       <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:10" ht="14.4">
-      <c r="A16" s="31"/>
+      <c r="A16" s="32"/>
       <c r="B16" s="5">
         <v>8</v>
       </c>
@@ -10107,7 +10187,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="14.4">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="35" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="9"/>
@@ -10119,7 +10199,7 @@
       <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:10" ht="14.4">
-      <c r="A18" s="31"/>
+      <c r="A18" s="32"/>
       <c r="B18" s="5">
         <v>11</v>
       </c>
@@ -10147,7 +10227,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="28.8">
-      <c r="A19" s="31"/>
+      <c r="A19" s="32"/>
       <c r="B19" s="5">
         <v>13</v>
       </c>
@@ -10159,7 +10239,7 @@
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:10" ht="28.8">
-      <c r="A20" s="31"/>
+      <c r="A20" s="32"/>
       <c r="B20" s="5">
         <v>14</v>
       </c>
@@ -10171,7 +10251,7 @@
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="14.4">
-      <c r="A21" s="31"/>
+      <c r="A21" s="32"/>
       <c r="B21" s="5">
         <v>15</v>
       </c>
@@ -10183,7 +10263,7 @@
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="31"/>
+      <c r="A22" s="32"/>
       <c r="B22" s="5">
         <v>16</v>
       </c>
@@ -10195,7 +10275,7 @@
       <c r="F22" s="8"/>
     </row>
     <row r="23" spans="1:10" ht="14.4">
-      <c r="A23" s="34" t="s">
+      <c r="A23" s="35" t="s">
         <v>20</v>
       </c>
       <c r="B23" s="9"/>
@@ -10207,7 +10287,7 @@
       <c r="F23" s="12"/>
     </row>
     <row r="24" spans="1:10" ht="28.8">
-      <c r="A24" s="31"/>
+      <c r="A24" s="32"/>
       <c r="B24" s="23">
         <v>17</v>
       </c>
@@ -10235,7 +10315,7 @@
       </c>
     </row>
     <row r="25" spans="1:10" ht="28.8">
-      <c r="A25" s="31"/>
+      <c r="A25" s="32"/>
       <c r="B25" s="5">
         <v>18</v>
       </c>
@@ -10247,7 +10327,7 @@
       <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:10" ht="14.4">
-      <c r="A26" s="31"/>
+      <c r="A26" s="32"/>
       <c r="B26" s="5">
         <v>19</v>
       </c>
@@ -10259,7 +10339,7 @@
       <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:10" ht="14.4">
-      <c r="A27" s="31"/>
+      <c r="A27" s="32"/>
       <c r="B27" s="5">
         <v>21</v>
       </c>
@@ -10271,7 +10351,7 @@
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="31"/>
+      <c r="A28" s="32"/>
       <c r="B28" s="5">
         <v>22</v>
       </c>
@@ -10283,7 +10363,7 @@
       <c r="F28" s="8"/>
     </row>
     <row r="29" spans="1:10" ht="14.4">
-      <c r="A29" s="42" t="s">
+      <c r="A29" s="43" t="s">
         <v>11</v>
       </c>
       <c r="B29" s="9"/>
@@ -10295,7 +10375,7 @@
       <c r="F29" s="12"/>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="42"/>
+      <c r="A30" s="43"/>
       <c r="B30" s="5">
         <v>24</v>
       </c>
@@ -10323,7 +10403,7 @@
       </c>
     </row>
     <row r="31" spans="1:10" ht="28.8">
-      <c r="A31" s="42"/>
+      <c r="A31" s="43"/>
       <c r="B31" s="5">
         <v>26</v>
       </c>
@@ -10335,7 +10415,7 @@
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="14.4">
-      <c r="A32" s="42"/>
+      <c r="A32" s="43"/>
       <c r="B32" s="5">
         <v>27</v>
       </c>
@@ -10347,7 +10427,7 @@
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="42"/>
+      <c r="A33" s="43"/>
       <c r="B33" s="5">
         <v>28</v>
       </c>
@@ -10359,7 +10439,7 @@
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="42"/>
+      <c r="A34" s="43"/>
       <c r="B34" s="5">
         <v>29</v>
       </c>
@@ -10371,7 +10451,7 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1">
-      <c r="A35" s="29" t="s">
+      <c r="A35" s="30" t="s">
         <v>30</v>
       </c>
       <c r="B35" s="9"/>
@@ -10383,7 +10463,7 @@
       <c r="F35" s="12"/>
     </row>
     <row r="36" spans="1:10" ht="28.8">
-      <c r="A36" s="30"/>
+      <c r="A36" s="31"/>
       <c r="B36" s="5">
         <v>30</v>
       </c>
@@ -10411,7 +10491,7 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="14.4">
-      <c r="A37" s="30"/>
+      <c r="A37" s="31"/>
       <c r="B37" s="5">
         <v>31</v>
       </c>
@@ -10423,7 +10503,7 @@
       <c r="F37" s="8"/>
     </row>
     <row r="38" spans="1:10" ht="28.8">
-      <c r="A38" s="30"/>
+      <c r="A38" s="31"/>
       <c r="B38" s="5">
         <v>32</v>
       </c>
@@ -10435,7 +10515,7 @@
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="14.4">
-      <c r="A39" s="30"/>
+      <c r="A39" s="31"/>
       <c r="B39" s="5"/>
       <c r="C39" s="8" t="s">
         <v>105</v>
@@ -10445,7 +10525,7 @@
       <c r="F39" s="8"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="30"/>
+      <c r="A40" s="31"/>
       <c r="B40" s="9"/>
       <c r="C40" s="10" t="s">
         <v>15</v>
@@ -10455,7 +10535,7 @@
       <c r="F40" s="12"/>
     </row>
     <row r="41" spans="1:10" ht="14.4">
-      <c r="A41" s="30"/>
+      <c r="A41" s="31"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
@@ -10483,7 +10563,7 @@
       </c>
     </row>
     <row r="42" spans="1:10" ht="14.4">
-      <c r="A42" s="30"/>
+      <c r="A42" s="31"/>
       <c r="B42" s="5">
         <v>34</v>
       </c>
@@ -10524,17 +10604,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:F3"/>
     <mergeCell ref="A5:A14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A17:A22"/>
     <mergeCell ref="A29:A34"/>
     <mergeCell ref="A35:A42"/>
     <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:F3"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D23 D15 D17 D40 D35 D29" xr:uid="{00000000-0002-0000-0300-000000000000}">
@@ -10564,41 +10644,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="33"/>
+      <c r="B2" s="34"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="40"/>
+      <c r="E2" s="41"/>
       <c r="F2" s="21" t="e">
         <f>COUNTIF(D5:D43,"Sim")/(COUNTA(D5:D43)-COUNTIF(D5:D43,"NA"))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="33"/>
+      <c r="B3" s="34"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="44"/>
-      <c r="F3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="46"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -10621,7 +10701,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="35" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -10633,7 +10713,7 @@
       <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="31"/>
+      <c r="A6" s="32"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -10661,7 +10741,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="14.4">
-      <c r="A7" s="31"/>
+      <c r="A7" s="32"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -10671,7 +10751,7 @@
       <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A8" s="31"/>
+      <c r="A8" s="32"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
@@ -10699,7 +10779,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="14.4">
-      <c r="A9" s="31"/>
+      <c r="A9" s="32"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10" t="s">
         <v>14</v>
@@ -10709,7 +10789,7 @@
       <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:10" ht="28.8">
-      <c r="A10" s="31"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="5">
         <v>3</v>
       </c>
@@ -10737,7 +10817,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.8">
-      <c r="A11" s="31"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="5">
         <v>4</v>
       </c>
@@ -10749,7 +10829,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="29.25" customHeight="1">
-      <c r="A12" s="31"/>
+      <c r="A12" s="32"/>
       <c r="B12" s="5">
         <v>5</v>
       </c>
@@ -10761,7 +10841,7 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="31"/>
+      <c r="A13" s="32"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>4</v>
@@ -10771,7 +10851,7 @@
       <c r="F13" s="12"/>
     </row>
     <row r="14" spans="1:10" ht="14.4">
-      <c r="A14" s="31"/>
+      <c r="A14" s="32"/>
       <c r="B14" s="5">
         <v>6</v>
       </c>
@@ -10799,7 +10879,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1">
-      <c r="A15" s="34" t="s">
+      <c r="A15" s="35" t="s">
         <v>18</v>
       </c>
       <c r="B15" s="9"/>
@@ -10811,7 +10891,7 @@
       <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:10" ht="14.4">
-      <c r="A16" s="31"/>
+      <c r="A16" s="32"/>
       <c r="B16" s="5">
         <v>8</v>
       </c>
@@ -10839,7 +10919,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="35" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="9"/>
@@ -10851,7 +10931,7 @@
       <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:10" ht="14.4">
-      <c r="A18" s="31"/>
+      <c r="A18" s="32"/>
       <c r="B18" s="5">
         <v>9</v>
       </c>
@@ -10879,7 +10959,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="14.4">
-      <c r="A19" s="31"/>
+      <c r="A19" s="32"/>
       <c r="B19" s="5">
         <v>10</v>
       </c>
@@ -10891,7 +10971,7 @@
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:10" ht="28.8">
-      <c r="A20" s="31"/>
+      <c r="A20" s="32"/>
       <c r="B20" s="5">
         <v>11</v>
       </c>
@@ -10903,7 +10983,7 @@
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="14.4">
-      <c r="A21" s="35"/>
+      <c r="A21" s="36"/>
       <c r="B21" s="5">
         <v>13</v>
       </c>
@@ -10915,7 +10995,7 @@
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="34" t="s">
+      <c r="A22" s="35" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="9"/>
@@ -10927,7 +11007,7 @@
       <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:10" ht="14.4">
-      <c r="A23" s="31"/>
+      <c r="A23" s="32"/>
       <c r="B23" s="5">
         <v>14</v>
       </c>
@@ -10955,7 +11035,7 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="14.4">
-      <c r="A24" s="31"/>
+      <c r="A24" s="32"/>
       <c r="B24" s="5">
         <v>15</v>
       </c>
@@ -10967,7 +11047,7 @@
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1">
-      <c r="A25" s="34" t="s">
+      <c r="A25" s="35" t="s">
         <v>21</v>
       </c>
       <c r="B25" s="9"/>
@@ -10979,7 +11059,7 @@
       <c r="F25" s="12"/>
     </row>
     <row r="26" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A26" s="31"/>
+      <c r="A26" s="32"/>
       <c r="B26" s="23">
         <v>24</v>
       </c>
@@ -11007,7 +11087,7 @@
       </c>
     </row>
     <row r="27" spans="1:10" s="1" customFormat="1" ht="43.2">
-      <c r="A27" s="31"/>
+      <c r="A27" s="32"/>
       <c r="B27" s="5">
         <v>25</v>
       </c>
@@ -11019,7 +11099,7 @@
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="31"/>
+      <c r="A28" s="32"/>
       <c r="B28" s="9"/>
       <c r="C28" s="10" t="s">
         <v>10</v>
@@ -11029,7 +11109,7 @@
       <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:10" ht="28.8">
-      <c r="A29" s="31"/>
+      <c r="A29" s="32"/>
       <c r="B29" s="23">
         <v>26</v>
       </c>
@@ -11057,7 +11137,7 @@
       </c>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="42" t="s">
+      <c r="A30" s="43" t="s">
         <v>11</v>
       </c>
       <c r="B30" s="9"/>
@@ -11069,7 +11149,7 @@
       <c r="F30" s="12"/>
     </row>
     <row r="31" spans="1:10" ht="14.4">
-      <c r="A31" s="42"/>
+      <c r="A31" s="43"/>
       <c r="B31" s="5">
         <v>19</v>
       </c>
@@ -11097,7 +11177,7 @@
       </c>
     </row>
     <row r="32" spans="1:10" ht="28.8">
-      <c r="A32" s="42"/>
+      <c r="A32" s="43"/>
       <c r="B32" s="5">
         <v>20</v>
       </c>
@@ -11109,7 +11189,7 @@
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="42"/>
+      <c r="A33" s="43"/>
       <c r="B33" s="5">
         <v>21</v>
       </c>
@@ -11121,7 +11201,7 @@
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="42"/>
+      <c r="A34" s="43"/>
       <c r="B34" s="5">
         <v>24</v>
       </c>
@@ -11133,7 +11213,7 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="14.4">
-      <c r="A35" s="42"/>
+      <c r="A35" s="43"/>
       <c r="B35" s="5">
         <v>25</v>
       </c>
@@ -11145,7 +11225,7 @@
       <c r="F35" s="8"/>
     </row>
     <row r="36" spans="1:10" ht="15" customHeight="1">
-      <c r="A36" s="29" t="s">
+      <c r="A36" s="30" t="s">
         <v>30</v>
       </c>
       <c r="B36" s="9"/>
@@ -11157,7 +11237,7 @@
       <c r="F36" s="12"/>
     </row>
     <row r="37" spans="1:10" ht="28.8">
-      <c r="A37" s="30"/>
+      <c r="A37" s="31"/>
       <c r="B37" s="5">
         <v>26</v>
       </c>
@@ -11185,7 +11265,7 @@
       </c>
     </row>
     <row r="38" spans="1:10" ht="14.4">
-      <c r="A38" s="30"/>
+      <c r="A38" s="31"/>
       <c r="B38" s="5">
         <v>27</v>
       </c>
@@ -11197,7 +11277,7 @@
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="28.8">
-      <c r="A39" s="30"/>
+      <c r="A39" s="31"/>
       <c r="B39" s="5">
         <v>28</v>
       </c>
@@ -11209,7 +11289,7 @@
       <c r="F39" s="8"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="30"/>
+      <c r="A40" s="31"/>
       <c r="B40" s="5"/>
       <c r="C40" s="8" t="s">
         <v>105</v>
@@ -11219,7 +11299,7 @@
       <c r="F40" s="8"/>
     </row>
     <row r="41" spans="1:10" ht="14.4">
-      <c r="A41" s="30"/>
+      <c r="A41" s="31"/>
       <c r="B41" s="9"/>
       <c r="C41" s="10" t="s">
         <v>15</v>
@@ -11229,7 +11309,7 @@
       <c r="F41" s="12"/>
     </row>
     <row r="42" spans="1:10" ht="14.4">
-      <c r="A42" s="30"/>
+      <c r="A42" s="31"/>
       <c r="B42" s="5">
         <v>29</v>
       </c>
@@ -11257,7 +11337,7 @@
       </c>
     </row>
     <row r="43" spans="1:10" ht="14.4">
-      <c r="A43" s="30"/>
+      <c r="A43" s="31"/>
       <c r="B43" s="5">
         <v>30</v>
       </c>
@@ -11298,11 +11378,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="A30:A35"/>
-    <mergeCell ref="A36:A43"/>
-    <mergeCell ref="A17:A21"/>
-    <mergeCell ref="A25:A29"/>
     <mergeCell ref="A5:A14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A1:F1"/>
@@ -11310,6 +11385,11 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="D3:F3"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A30:A35"/>
+    <mergeCell ref="A36:A43"/>
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="A25:A29"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D25 D17 D15 D22 D41 D36 D30 D28" xr:uid="{00000000-0002-0000-0400-000000000000}">

</xml_diff>